<commit_message>
docs: consolidate UHMR readiness and configurable activation with technical basis
</commit_message>
<xml_diff>
--- a/05_PLANILHA_DIMENSIONAMENTO_CUSTOS_UHMR.xlsx
+++ b/05_PLANILHA_DIMENSIONAMENTO_CUSTOS_UHMR.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rccaeaaffe7bd4881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="2" r:id="R53dc976c8f764557"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveis" sheetId="3" r:id="Rc267827d04df4714"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custos" sheetId="4" r:id="Ra1097492cef941d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cenarios" sheetId="5" r:id="Rc9e9e65fb54d431c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipes" sheetId="6" r:id="Re72913eec47a4f4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipamentos" sheetId="7" r:id="R2d5219a5f7fe4439"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLA" sheetId="8" r:id="R9e116e9135ec4679"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscos" sheetId="9" r:id="Ra48d245b0aad4d85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Estado" sheetId="10" r:id="Rad7b75a20d7e4a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendencias" sheetId="11" r:id="Ree952061e7c1464a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="12" r:id="Rc68753e2f6d94179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R30a3710acda14dc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="2" r:id="R3a932abfe84d4ea3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveis" sheetId="3" r:id="R5bb887e00d4144df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custos" sheetId="4" r:id="R251e92f2c9554fe3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cenarios" sheetId="5" r:id="Rb3971835b58b4fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipes" sheetId="6" r:id="Rff2e21c0dc9a4789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipamentos" sheetId="7" r:id="R073bbafe1e3846d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLA" sheetId="8" r:id="R5d69c85457c44c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscos" sheetId="9" r:id="Rccf5171a44b64814"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dados Estado" sheetId="10" r:id="R8934f9d1d0204f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pendencias" sheetId="11" r:id="Rbd08f5de92bc4d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fontes" sheetId="12" r:id="R75194dcbf7964754"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acionamento" sheetId="13" r:id="R8d545b22e7a14aea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,11 +25,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="R$ #,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="0.0%"/>
+    <x:numFmt numFmtId="202" formatCode="&quot;R$&quot; #,##0.00"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -72,8 +74,39 @@
       <x:color rgb="FF000000"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF003966"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -93,6 +126,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7EEF5"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -151,7 +199,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -240,6 +288,46 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -251,7 +339,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -261,7 +349,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -271,7 +359,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -281,7 +369,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -601,8 +689,7 @@
         <x:v>Custo anual estimado</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:f>IFERROR(INDEX(Cenarios!$J$7:$J$10,MATCH(B7,Cenarios!$A$7:$A$10,0)),"PENDENTE")</x:f>
-        <x:v>PENDENTE</x:v>
+        <x:f>IFERROR(INDEX(Cenarios!$J$6:$J$9,MATCH(B7,Cenarios!$A$6:$A$9,0)),"PENDENTE")</x:f>
       </x:c>
       <x:c r="C8" s="34"/>
       <x:c r="D8" s="34"/>
@@ -616,7 +703,7 @@
         <x:v>Itens de custo pendentes</x:v>
       </x:c>
       <x:c r="B9" s="21" t="n">
-        <x:f>COUNTBLANK(Custos!$D$7:$D$16)</x:f>
+        <x:f>COUNTBLANK(Custos!$D$6:$D$15)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="C9" s="34"/>
@@ -835,10 +922,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="35" t="str">
-        <x:v>1. Preencha Premissas, Custos, Equipes e Equipamentos.
-2. Defina a frequência dos cenários.
-3. Atualize dados estaduais e decisões.
-4. Revise os resultados antes de incorporar valores ao ETP, TR, edital ou contrato.</x:v>
+        <x:v>1. Preencha custos e fontes.
+2. Use Acionamento para a configuração efetiva, inclusive só medicamentos.
+3. N0 remunera disponibilidade comprovada e manutenção pela empresa.
+4. A OA depende do Secretário, com análise de risco e cenários.</x:v>
       </x:c>
       <x:c r="B21" s="35"/>
       <x:c r="C21" s="35"/>
@@ -2088,6 +2175,792 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF003966"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="40" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="38" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="36" t="str">
+        <x:v>Configuração da missão UHMR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="40" t="str">
+        <x:v>Revisão</x:v>
+      </x:c>
+      <x:c r="B3" s="40" t="str">
+        <x:v>2.1 — 28/09/2026</x:v>
+      </x:c>
+      <x:c r="C3" s="40"/>
+      <x:c r="D3" s="40"/>
+      <x:c r="E3" s="40"/>
+      <x:c r="F3" s="40"/>
+      <x:c r="G3" s="40"/>
+      <x:c r="H3" s="40"/>
+      <x:c r="I3" s="40"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="40" t="str">
+        <x:v>Modalidade da missão</x:v>
+      </x:c>
+      <x:c r="B4" s="41" t="str">
+        <x:v>A definir</x:v>
+      </x:c>
+      <x:c r="C4" s="40"/>
+      <x:c r="D4" s="40"/>
+      <x:c r="E4" s="40"/>
+      <x:c r="F4" s="40"/>
+      <x:c r="G4" s="40"/>
+      <x:c r="H4" s="40"/>
+      <x:c r="I4" s="40"/>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="A5" s="40" t="str">
+        <x:v>Nível de referência</x:v>
+      </x:c>
+      <x:c r="B5" s="41" t="str">
+        <x:v>Não obrigatório</x:v>
+      </x:c>
+      <x:c r="C5" s="40"/>
+      <x:c r="D5" s="40"/>
+      <x:c r="E5" s="40"/>
+      <x:c r="F5" s="40"/>
+      <x:c r="G5" s="40"/>
+      <x:c r="H5" s="40"/>
+      <x:c r="I5" s="40"/>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="40" t="str">
+        <x:v>Nota técnica e risco</x:v>
+      </x:c>
+      <x:c r="B6" s="41"/>
+      <x:c r="C6" s="40"/>
+      <x:c r="D6" s="40"/>
+      <x:c r="E6" s="40"/>
+      <x:c r="F6" s="40"/>
+      <x:c r="G6" s="40"/>
+      <x:c r="H6" s="40"/>
+      <x:c r="I6" s="40"/>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="A7" s="40" t="str">
+        <x:v>Cenários e capacidade da rede</x:v>
+      </x:c>
+      <x:c r="B7" s="41"/>
+      <x:c r="C7" s="40"/>
+      <x:c r="D7" s="40"/>
+      <x:c r="E7" s="40"/>
+      <x:c r="F7" s="40"/>
+      <x:c r="G7" s="40"/>
+      <x:c r="H7" s="40"/>
+      <x:c r="I7" s="40"/>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="A8" s="40" t="str">
+        <x:v>OA e decisão do Secretário</x:v>
+      </x:c>
+      <x:c r="B8" s="41"/>
+      <x:c r="C8" s="40"/>
+      <x:c r="D8" s="40"/>
+      <x:c r="E8" s="40"/>
+      <x:c r="F8" s="40"/>
+      <x:c r="G8" s="40"/>
+      <x:c r="H8" s="40"/>
+      <x:c r="I8" s="40"/>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="40" t="str">
+        <x:v>Destino e prazo</x:v>
+      </x:c>
+      <x:c r="B9" s="41"/>
+      <x:c r="C9" s="40"/>
+      <x:c r="D9" s="40"/>
+      <x:c r="E9" s="40"/>
+      <x:c r="F9" s="40"/>
+      <x:c r="G9" s="40"/>
+      <x:c r="H9" s="40"/>
+      <x:c r="I9" s="40"/>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="A10" s="40" t="str">
+        <x:v>Dependências e responsáveis</x:v>
+      </x:c>
+      <x:c r="B10" s="41"/>
+      <x:c r="C10" s="40"/>
+      <x:c r="D10" s="40"/>
+      <x:c r="E10" s="40"/>
+      <x:c r="F10" s="40"/>
+      <x:c r="G10" s="40"/>
+      <x:c r="H10" s="40"/>
+      <x:c r="I10" s="40"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="40" t="str">
+        <x:v>Meses de prontidão</x:v>
+      </x:c>
+      <x:c r="B11" s="41" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C11" s="40"/>
+      <x:c r="D11" s="40"/>
+      <x:c r="E11" s="40"/>
+      <x:c r="F11" s="40"/>
+      <x:c r="G11" s="40"/>
+      <x:c r="H11" s="40"/>
+      <x:c r="I11" s="40"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="40" t="str">
+        <x:v>Mensalidade N0</x:v>
+      </x:c>
+      <x:c r="B12" s="49" t="str">
+        <x:f>IF(Custos!D6="","",Custos!D6)</x:f>
+      </x:c>
+      <x:c r="C12" s="40"/>
+      <x:c r="D12" s="40"/>
+      <x:c r="E12" s="40"/>
+      <x:c r="F12" s="40"/>
+      <x:c r="G12" s="40"/>
+      <x:c r="H12" s="40"/>
+      <x:c r="I12" s="40"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="40"/>
+      <x:c r="B13" s="40"/>
+      <x:c r="C13" s="40"/>
+      <x:c r="D13" s="40"/>
+      <x:c r="E13" s="40"/>
+      <x:c r="F13" s="40"/>
+      <x:c r="G13" s="40"/>
+      <x:c r="H13" s="40"/>
+      <x:c r="I13" s="40"/>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="45" t="str">
+        <x:v>Item ou módulo</x:v>
+      </x:c>
+      <x:c r="B14" s="45" t="str">
+        <x:v>Unidade</x:v>
+      </x:c>
+      <x:c r="C14" s="45" t="str">
+        <x:v>Quantidade</x:v>
+      </x:c>
+      <x:c r="D14" s="45" t="str">
+        <x:v>Períodos</x:v>
+      </x:c>
+      <x:c r="E14" s="45" t="str">
+        <x:v>Preço unitário</x:v>
+      </x:c>
+      <x:c r="F14" s="45" t="str">
+        <x:v>Incluído no N0</x:v>
+      </x:c>
+      <x:c r="G14" s="45" t="str">
+        <x:v>Subtotal R$</x:v>
+      </x:c>
+      <x:c r="H14" s="45" t="str">
+        <x:v>Situação</x:v>
+      </x:c>
+      <x:c r="I14" s="45" t="str">
+        <x:v>Fonte e escopo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="38" customHeight="1">
+      <x:c r="A15" s="46" t="str">
+        <x:v>Leitos</x:v>
+      </x:c>
+      <x:c r="B15" s="46" t="str">
+        <x:v>leito-dia</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E15" s="50"/>
+      <x:c r="F15" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G15" s="51" t="n">
+        <x:f>IF(C15=0,0,IF(OR(C15&lt;0,D15&lt;=0,E15&lt;0),"",IF(F15="Sim",0,IF(OR(E15="",D15=""),"",C15*D15*E15))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="42" t="str">
+        <x:f>IF(C15=0,"Não acionado",IF(OR(C15&lt;0,D15&lt;=0,E15&lt;0),"Rever valores",IF(F15="Sim","Já incluído",IF(OR(E15="",D15=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I15" s="46"/>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" s="46" t="str">
+        <x:v>Laboratório</x:v>
+      </x:c>
+      <x:c r="B16" s="46" t="str">
+        <x:v>módulo-dia</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E16" s="50"/>
+      <x:c r="F16" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G16" s="51" t="n">
+        <x:f>IF(C16=0,0,IF(OR(C16&lt;0,D16&lt;=0,E16&lt;0),"",IF(F16="Sim",0,IF(OR(E16="",D16=""),"",C16*D16*E16))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="42" t="str">
+        <x:f>IF(C16=0,"Não acionado",IF(OR(C16&lt;0,D16&lt;=0,E16&lt;0),"Rever valores",IF(F16="Sim","Já incluído",IF(OR(E16="",D16=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I16" s="46"/>
+    </x:row>
+    <x:row r="17" ht="38" customHeight="1">
+      <x:c r="A17" s="46" t="str">
+        <x:v>Medicamento — discriminar</x:v>
+      </x:c>
+      <x:c r="B17" s="46" t="str">
+        <x:v>unidade</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E17" s="50"/>
+      <x:c r="F17" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G17" s="51" t="n">
+        <x:f>IF(C17=0,0,IF(OR(C17&lt;0,D17&lt;=0,E17&lt;0),"",IF(F17="Sim",0,IF(OR(E17="",D17=""),"",C17*D17*E17))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="42" t="str">
+        <x:f>IF(C17=0,"Não acionado",IF(OR(C17&lt;0,D17&lt;=0,E17&lt;0),"Rever valores",IF(F17="Sim","Já incluído",IF(OR(E17="",D17=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I17" s="46"/>
+    </x:row>
+    <x:row r="18" ht="38" customHeight="1">
+      <x:c r="A18" s="46" t="str">
+        <x:v>Insumo — discriminar</x:v>
+      </x:c>
+      <x:c r="B18" s="46" t="str">
+        <x:v>unidade</x:v>
+      </x:c>
+      <x:c r="C18" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E18" s="50"/>
+      <x:c r="F18" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G18" s="51" t="n">
+        <x:f>IF(C18=0,0,IF(OR(C18&lt;0,D18&lt;=0,E18&lt;0),"",IF(F18="Sim",0,IF(OR(E18="",D18=""),"",C18*D18*E18))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="42" t="str">
+        <x:f>IF(C18=0,"Não acionado",IF(OR(C18&lt;0,D18&lt;=0,E18&lt;0),"Rever valores",IF(F18="Sim","Já incluído",IF(OR(E18="",D18=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I18" s="46"/>
+    </x:row>
+    <x:row r="19" ht="38" customHeight="1">
+      <x:c r="A19" s="46" t="str">
+        <x:v>Transporte</x:v>
+      </x:c>
+      <x:c r="B19" s="46" t="str">
+        <x:v>evento</x:v>
+      </x:c>
+      <x:c r="C19" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D19" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="50"/>
+      <x:c r="F19" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G19" s="51" t="n">
+        <x:f>IF(C19=0,0,IF(OR(C19&lt;0,D19&lt;=0,E19&lt;0),"",IF(F19="Sim",0,IF(OR(E19="",D19=""),"",C19*D19*E19))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="42" t="str">
+        <x:f>IF(C19=0,"Não acionado",IF(OR(C19&lt;0,D19&lt;=0,E19&lt;0),"Rever valores",IF(F19="Sim","Já incluído",IF(OR(E19="",D19=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I19" s="46"/>
+    </x:row>
+    <x:row r="20" ht="38" customHeight="1">
+      <x:c r="A20" s="46" t="str">
+        <x:v>Implantação</x:v>
+      </x:c>
+      <x:c r="B20" s="46" t="str">
+        <x:v>evento</x:v>
+      </x:c>
+      <x:c r="C20" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="50"/>
+      <x:c r="F20" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G20" s="51" t="n">
+        <x:f>IF(C20=0,0,IF(OR(C20&lt;0,D20&lt;=0,E20&lt;0),"",IF(F20="Sim",0,IF(OR(E20="",D20=""),"",C20*D20*E20))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="42" t="str">
+        <x:f>IF(C20=0,"Não acionado",IF(OR(C20&lt;0,D20&lt;=0,E20&lt;0),"Rever valores",IF(F20="Sim","Já incluído",IF(OR(E20="",D20=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I20" s="46"/>
+    </x:row>
+    <x:row r="21" ht="38" customHeight="1">
+      <x:c r="A21" s="46" t="str">
+        <x:v>Equipe</x:v>
+      </x:c>
+      <x:c r="B21" s="46" t="str">
+        <x:v>equipe-dia</x:v>
+      </x:c>
+      <x:c r="C21" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E21" s="50"/>
+      <x:c r="F21" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G21" s="51" t="n">
+        <x:f>IF(C21=0,0,IF(OR(C21&lt;0,D21&lt;=0,E21&lt;0),"",IF(F21="Sim",0,IF(OR(E21="",D21=""),"",C21*D21*E21))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="42" t="str">
+        <x:f>IF(C21=0,"Não acionado",IF(OR(C21&lt;0,D21&lt;=0,E21&lt;0),"Rever valores",IF(F21="Sim","Já incluído",IF(OR(E21="",D21=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I21" s="46"/>
+    </x:row>
+    <x:row r="22" ht="38" customHeight="1">
+      <x:c r="A22" s="46" t="str">
+        <x:v>Suporte compartilhado</x:v>
+      </x:c>
+      <x:c r="B22" s="46" t="str">
+        <x:v>módulo-dia</x:v>
+      </x:c>
+      <x:c r="C22" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E22" s="50"/>
+      <x:c r="F22" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G22" s="51" t="n">
+        <x:f>IF(C22=0,0,IF(OR(C22&lt;0,D22&lt;=0,E22&lt;0),"",IF(F22="Sim",0,IF(OR(E22="",D22=""),"",C22*D22*E22))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="42" t="str">
+        <x:f>IF(C22=0,"Não acionado",IF(OR(C22&lt;0,D22&lt;=0,E22&lt;0),"Rever valores",IF(F22="Sim","Já incluído",IF(OR(E22="",D22=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I22" s="46"/>
+    </x:row>
+    <x:row r="23" ht="38" customHeight="1">
+      <x:c r="A23" s="46" t="str">
+        <x:v>Desmobilização</x:v>
+      </x:c>
+      <x:c r="B23" s="46" t="str">
+        <x:v>evento</x:v>
+      </x:c>
+      <x:c r="C23" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E23" s="50"/>
+      <x:c r="F23" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G23" s="51" t="n">
+        <x:f>IF(C23=0,0,IF(OR(C23&lt;0,D23&lt;=0,E23&lt;0),"",IF(F23="Sim",0,IF(OR(E23="",D23=""),"",C23*D23*E23))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="42" t="str">
+        <x:f>IF(C23=0,"Não acionado",IF(OR(C23&lt;0,D23&lt;=0,E23&lt;0),"Rever valores",IF(F23="Sim","Já incluído",IF(OR(E23="",D23=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I23" s="46"/>
+    </x:row>
+    <x:row r="24" ht="38" customHeight="1">
+      <x:c r="A24" s="53" t="str">
+        <x:v>Manutenção ordinária</x:v>
+      </x:c>
+      <x:c r="B24" s="53" t="str">
+        <x:v>incluída</x:v>
+      </x:c>
+      <x:c r="C24" s="54" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D24" s="54" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E24" s="55" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="53" t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c r="G24" s="51" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="42" t="str">
+        <x:v>Incluída no N0</x:v>
+      </x:c>
+      <x:c r="I24" s="46" t="str">
+        <x:v>Custeada pela empresa</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="38" customHeight="1">
+      <x:c r="A25" s="46" t="str">
+        <x:v>Item adicional 1</x:v>
+      </x:c>
+      <x:c r="B25" s="46" t="str">
+        <x:v>unidade</x:v>
+      </x:c>
+      <x:c r="C25" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D25" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E25" s="50"/>
+      <x:c r="F25" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G25" s="51" t="n">
+        <x:f>IF(C25=0,0,IF(OR(C25&lt;0,D25&lt;=0,E25&lt;0),"",IF(F25="Sim",0,IF(OR(E25="",D25=""),"",C25*D25*E25))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H25" s="42" t="str">
+        <x:f>IF(C25=0,"Não acionado",IF(OR(C25&lt;0,D25&lt;=0,E25&lt;0),"Rever valores",IF(F25="Sim","Já incluído",IF(OR(E25="",D25=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I25" s="46"/>
+    </x:row>
+    <x:row r="26" ht="38" customHeight="1">
+      <x:c r="A26" s="46" t="str">
+        <x:v>Item adicional 2</x:v>
+      </x:c>
+      <x:c r="B26" s="46" t="str">
+        <x:v>unidade</x:v>
+      </x:c>
+      <x:c r="C26" s="47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D26" s="47" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="50"/>
+      <x:c r="F26" s="46" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="G26" s="51" t="n">
+        <x:f>IF(C26=0,0,IF(OR(C26&lt;0,D26&lt;=0,E26&lt;0),"",IF(F26="Sim",0,IF(OR(E26="",D26=""),"",C26*D26*E26))))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H26" s="42" t="str">
+        <x:f>IF(C26=0,"Não acionado",IF(OR(C26&lt;0,D26&lt;=0,E26&lt;0),"Rever valores",IF(F26="Sim","Já incluído",IF(OR(E26="",D26=""),"Preço/período pendente","Calculado"))))</x:f>
+        <x:v>Não acionado</x:v>
+      </x:c>
+      <x:c r="I26" s="46"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="40"/>
+      <x:c r="B27" s="40"/>
+      <x:c r="C27" s="40"/>
+      <x:c r="D27" s="40"/>
+      <x:c r="E27" s="40"/>
+      <x:c r="F27" s="40"/>
+      <x:c r="G27" s="40"/>
+      <x:c r="H27" s="40"/>
+      <x:c r="I27" s="40"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="48" t="str">
+        <x:v>Custo variável da missão</x:v>
+      </x:c>
+      <x:c r="B28" s="52" t="n">
+        <x:f>IF(COUNT(G15:G26)&lt;12,"PENDENTE",SUM(G15:G26))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C28" s="40"/>
+      <x:c r="D28" s="40"/>
+      <x:c r="E28" s="40"/>
+      <x:c r="F28" s="40"/>
+      <x:c r="G28" s="40"/>
+      <x:c r="H28" s="40"/>
+      <x:c r="I28" s="40"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="48" t="str">
+        <x:v>Custo N0 no período</x:v>
+      </x:c>
+      <x:c r="B29" s="52" t="str">
+        <x:f>IF(OR(B11="",B12=""),"PENDENTE",B11*B12)</x:f>
+        <x:v>PENDENTE</x:v>
+      </x:c>
+      <x:c r="C29" s="40"/>
+      <x:c r="D29" s="40"/>
+      <x:c r="E29" s="40"/>
+      <x:c r="F29" s="40"/>
+      <x:c r="G29" s="40"/>
+      <x:c r="H29" s="40"/>
+      <x:c r="I29" s="40"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="48" t="str">
+        <x:v>Total estimado</x:v>
+      </x:c>
+      <x:c r="B30" s="52" t="str">
+        <x:f>IF(COUNT(B28:B29)&lt;2,"PENDENTE",SUM(B28:B29))</x:f>
+        <x:v>PENDENTE</x:v>
+      </x:c>
+      <x:c r="C30" s="40"/>
+      <x:c r="D30" s="40"/>
+      <x:c r="E30" s="40"/>
+      <x:c r="F30" s="40"/>
+      <x:c r="G30" s="40"/>
+      <x:c r="H30" s="40"/>
+      <x:c r="I30" s="40"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="40" t="str">
+        <x:v>Itens acionados sem cálculo</x:v>
+      </x:c>
+      <x:c r="B31" s="40" t="n">
+        <x:f>12-COUNT(G15:G26)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C31" s="40"/>
+      <x:c r="D31" s="40"/>
+      <x:c r="E31" s="40"/>
+      <x:c r="F31" s="40"/>
+      <x:c r="G31" s="40"/>
+      <x:c r="H31" s="40"/>
+      <x:c r="I31" s="40"/>
+    </x:row>
+    <x:row r="32" ht="40" customHeight="1">
+      <x:c r="A32" s="40" t="str">
+        <x:v>Instrução para autorização</x:v>
+      </x:c>
+      <x:c r="B32" s="42" t="str">
+        <x:f>IF(OR(B4="A definir",COUNTBLANK(B6:B10)&gt;0),"PENDENTE","Documentos informados; conferir ato")</x:f>
+        <x:v>PENDENTE</x:v>
+      </x:c>
+      <x:c r="C32" s="40"/>
+      <x:c r="D32" s="40"/>
+      <x:c r="E32" s="40"/>
+      <x:c r="F32" s="40"/>
+      <x:c r="G32" s="40"/>
+      <x:c r="H32" s="40"/>
+      <x:c r="I32" s="40"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="40"/>
+      <x:c r="B33" s="40"/>
+      <x:c r="C33" s="40"/>
+      <x:c r="D33" s="40"/>
+      <x:c r="E33" s="40"/>
+      <x:c r="F33" s="40"/>
+      <x:c r="G33" s="40"/>
+      <x:c r="H33" s="40"/>
+      <x:c r="I33" s="40"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="40" t="str">
+        <x:v>Regras de preenchimento</x:v>
+      </x:c>
+      <x:c r="B34" s="40"/>
+      <x:c r="C34" s="40"/>
+      <x:c r="D34" s="40"/>
+      <x:c r="E34" s="40"/>
+      <x:c r="F34" s="40"/>
+      <x:c r="G34" s="40"/>
+      <x:c r="H34" s="40"/>
+      <x:c r="I34" s="40"/>
+    </x:row>
+    <x:row r="35" ht="30" customHeight="1">
+      <x:c r="A35" s="42" t="str">
+        <x:v>N0 é remunerado mesmo sem uso, mediante disponibilidade comprovada. Manutenção ordinária está incluída nos preços.</x:v>
+      </x:c>
+      <x:c r="B35" s="42"/>
+      <x:c r="C35" s="42"/>
+      <x:c r="D35" s="42"/>
+      <x:c r="E35" s="42"/>
+      <x:c r="F35" s="42"/>
+      <x:c r="G35" s="42"/>
+      <x:c r="H35" s="42"/>
+      <x:c r="I35" s="42"/>
+    </x:row>
+    <x:row r="36" ht="30" customHeight="1">
+      <x:c r="A36" s="42" t="str">
+        <x:v>N1 a N4 são referenciais. Quantidade zero significa item não acionado. Preço vazio mantém o cálculo pendente.</x:v>
+      </x:c>
+      <x:c r="B36" s="42"/>
+      <x:c r="C36" s="42"/>
+      <x:c r="D36" s="42"/>
+      <x:c r="E36" s="42"/>
+      <x:c r="F36" s="42"/>
+      <x:c r="G36" s="42"/>
+      <x:c r="H36" s="42"/>
+      <x:c r="I36" s="42"/>
+    </x:row>
+    <x:row r="37" ht="30" customHeight="1">
+      <x:c r="A37" s="42" t="str">
+        <x:v>Em leito-dia ou módulo-dia, informe unidades em Quantidade e dias em Períodos. Fornecimento unitário usa Períodos = 1.</x:v>
+      </x:c>
+      <x:c r="B37" s="42"/>
+      <x:c r="C37" s="42"/>
+      <x:c r="D37" s="42"/>
+      <x:c r="E37" s="42"/>
+      <x:c r="F37" s="42"/>
+      <x:c r="G37" s="42"/>
+      <x:c r="H37" s="42"/>
+      <x:c r="I37" s="42"/>
+    </x:row>
+    <x:row r="38" ht="30" customHeight="1">
+      <x:c r="A38" s="42" t="str">
+        <x:v>Dez leitos: selecione leitos e suportes necessários. Laboratório isolado: selecione laboratório e suas dependências.</x:v>
+      </x:c>
+      <x:c r="B38" s="42"/>
+      <x:c r="C38" s="42"/>
+      <x:c r="D38" s="42"/>
+      <x:c r="E38" s="42"/>
+      <x:c r="F38" s="42"/>
+      <x:c r="G38" s="42"/>
+      <x:c r="H38" s="42"/>
+      <x:c r="I38" s="42"/>
+    </x:row>
+    <x:row r="39" ht="30" customHeight="1">
+      <x:c r="A39" s="42" t="str">
+        <x:v>Medicamentos isolados: discrimine apresentação e unidade, quantidade, fonte do preço, conservação e entrega. Não selecione montagem inexistente.</x:v>
+      </x:c>
+      <x:c r="B39" s="42"/>
+      <x:c r="C39" s="42"/>
+      <x:c r="D39" s="42"/>
+      <x:c r="E39" s="42"/>
+      <x:c r="F39" s="42"/>
+      <x:c r="G39" s="42"/>
+      <x:c r="H39" s="42"/>
+      <x:c r="I39" s="42"/>
+    </x:row>
+    <x:row r="40" ht="30" customHeight="1">
+      <x:c r="A40" s="42" t="str">
+        <x:v>Não duplique suportes. Marque Incluído no N0 quando já remunerado. Para item incluso, o subtotal variável é zero.</x:v>
+      </x:c>
+      <x:c r="B40" s="42"/>
+      <x:c r="C40" s="42"/>
+      <x:c r="D40" s="42"/>
+      <x:c r="E40" s="42"/>
+      <x:c r="F40" s="42"/>
+      <x:c r="G40" s="42"/>
+      <x:c r="H40" s="42"/>
+      <x:c r="I40" s="42"/>
+    </x:row>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="42" t="str">
+        <x:v>A autorização cabe ao Secretário com documentação, risco e cenários. Documentos informados não significam autorização concedida.</x:v>
+      </x:c>
+      <x:c r="B41" s="42"/>
+      <x:c r="C41" s="42"/>
+      <x:c r="D41" s="42"/>
+      <x:c r="E41" s="42"/>
+      <x:c r="F41" s="42"/>
+      <x:c r="G41" s="42"/>
+      <x:c r="H41" s="42"/>
+      <x:c r="I41" s="42"/>
+    </x:row>
+    <x:row r="42" ht="30" customHeight="1">
+      <x:c r="A42" s="42" t="str">
+        <x:v>Esta aba estima uma missão. Para múltiplas missões, some parcelas variáveis e conte o N0 somente uma vez no mesmo período.</x:v>
+      </x:c>
+      <x:c r="B42" s="42"/>
+      <x:c r="C42" s="42"/>
+      <x:c r="D42" s="42"/>
+      <x:c r="E42" s="42"/>
+      <x:c r="F42" s="42"/>
+      <x:c r="G42" s="42"/>
+      <x:c r="H42" s="42"/>
+      <x:c r="I42" s="42"/>
+    </x:row>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="42" t="str">
+        <x:v>Fonte das premissas: orientação de projeto de 28/09/2026. Preços devem ter pesquisa e validação antes da contratação.</x:v>
+      </x:c>
+      <x:c r="B43" s="42"/>
+      <x:c r="C43" s="42"/>
+      <x:c r="D43" s="42"/>
+      <x:c r="E43" s="42"/>
+      <x:c r="F43" s="42"/>
+      <x:c r="G43" s="42"/>
+      <x:c r="H43" s="42"/>
+      <x:c r="I43" s="42"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A35:I35"/>
+    <x:mergeCell ref="A36:I36"/>
+    <x:mergeCell ref="A37:I37"/>
+    <x:mergeCell ref="A38:I38"/>
+    <x:mergeCell ref="A39:I39"/>
+    <x:mergeCell ref="A40:I40"/>
+    <x:mergeCell ref="A41:I41"/>
+    <x:mergeCell ref="A42:I42"/>
+    <x:mergeCell ref="A43:I43"/>
+  </x:mergeCells>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="F15:F26">
+      <x:formula1>"Sim,Não"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B4">
+      <x:formula1>"A definir,Sem ativação,Dez leitos,Laboratório isolado,Medicamentos isolados,Configuração mista"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr>
@@ -2447,7 +3320,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="33" t="str">
-        <x:v>Capacidades de referência. Quantitativos finais devem ser confirmados no dimensionamento.</x:v>
+        <x:v>N0 remunerado sem uso. N1–N4 são referências independentes. Dimensione a missão na aba Acionamento.</x:v>
       </x:c>
       <x:c r="B3" s="33"/>
       <x:c r="C3" s="33"/>
@@ -2542,7 +3415,7 @@
         <x:v>Comando, triagem, estabilização, consulta e POC</x:v>
       </x:c>
       <x:c r="H7" s="21" t="str">
-        <x:v>Definido</x:v>
+        <x:v>Referência</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2565,10 +3438,10 @@
         <x:v>Até 18 h</x:v>
       </x:c>
       <x:c r="G8" s="21" t="str">
-        <x:v>N1, internação, imagem e isolamento acionável</x:v>
+        <x:v>Internação, imagem e isolamento selecionáveis</x:v>
       </x:c>
       <x:c r="H8" s="21" t="str">
-        <x:v>Definido</x:v>
+        <x:v>Referência</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2594,7 +3467,7 @@
         <x:v>EMT Tipo 2 funcional, CME, RX, USG e WASH</x:v>
       </x:c>
       <x:c r="H9" s="21" t="str">
-        <x:v>Definido</x:v>
+        <x:v>Referência</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2669,7 +3542,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="33" t="str">
-        <x:v>Preços unitários são entradas. Subtotais e total são calculados automaticamente.</x:v>
+        <x:v>N0 inclui manutenção ordinária pela empresa. Para composição por itens e medicamentos isolados, use Acionamento.</x:v>
       </x:c>
       <x:c r="B3" s="33"/>
       <x:c r="C3" s="33"/>
@@ -2775,7 +3648,7 @@
         <x:v>Instalação</x:v>
       </x:c>
       <x:c r="C9" s="21" t="str">
-        <x:v>nível</x:v>
+        <x:v>configuração</x:v>
       </x:c>
       <x:c r="D9" s="28"/>
       <x:c r="E9" s="28"/>
@@ -2903,9 +3776,9 @@
       <x:c r="C16" s="29" t="str"/>
       <x:c r="D16" s="30"/>
       <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30" t="n">
-        <x:f>SUM(F6:F15)</x:f>
-        <x:v>0</x:v>
+      <x:c r="F16" s="30" t="str">
+        <x:f>IF(COUNTBLANK(D6:D15)&gt;0,"PENDENTE",SUM(F6:F15))</x:f>
+        <x:v>PENDENTE</x:v>
       </x:c>
       <x:c r="G16" s="29" t="str"/>
       <x:c r="H16" s="34"/>
@@ -2963,7 +3836,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="33" t="str">
-        <x:v>Frequências e durações são entradas de planejamento. Não representam histórico observado até serem substituídas por dados estaduais.</x:v>
+        <x:v>Cenários integrais de referência. Use Acionamento para módulos isolados. Preços não pesquisados permanecem pendentes.</x:v>
       </x:c>
       <x:c r="B3" s="33"/>
       <x:c r="C3" s="33"/>
@@ -3526,7 +4399,7 @@
         <x:v>Conteúdo funcional</x:v>
       </x:c>
       <x:c r="D5" s="17" t="str">
-        <x:v>Nível mínimo</x:v>
+        <x:v>Nível de referência</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
         <x:v>Quantidade</x:v>

</xml_diff>